<commit_message>
Float and signed working
</commit_message>
<xml_diff>
--- a/config/Map_Escepar_1729509304301.xlsx
+++ b/config/Map_Escepar_1729509304301.xlsx
@@ -474,32 +474,32 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Read_30115</t>
+          <t>ReadF32_41044</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>Read_30116</t>
+          <t>ReadF32_41046</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>Read_30117</t>
+          <t>WriteF32_41048</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>Read_30118</t>
+          <t>Write_41050</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>Mask_40000</t>
+          <t>Read_41050</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>Mask_41008</t>
+          <t>ReadS16_41050</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
@@ -562,17 +562,21 @@
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>0xFFFC 0x0002</t>
-        </is>
-      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>-522.0</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>3.0</t>
         </is>
       </c>
     </row>
@@ -630,17 +634,21 @@
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>0xFFFC 0x0002</t>
-        </is>
-      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>-522.1</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>3.0</t>
         </is>
       </c>
     </row>
@@ -690,22 +698,46 @@
           <t>Controller</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>4139.0</t>
+        </is>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1.1</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0.4363323152065277</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>0.2617993950843811</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>0xFFFC 0x0002</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr"/>
+          <t>65014.0</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>-522.0</t>
+        </is>
+      </c>
       <c r="R4" t="inlineStr">
         <is>
           <t>1.0</t>
@@ -766,17 +798,21 @@
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>0xFFFC 0x0002</t>
-        </is>
-      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>-522.3</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>2.0</t>
         </is>
       </c>
     </row>
@@ -826,25 +862,49 @@
           <t>Controller</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>4139.0</t>
+        </is>
+      </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>1.2</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2.169474251394558e-19</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2.169474251394558e-19</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>0xFFFC 0x0002</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr"/>
+          <t>4139.0</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>26355.0</t>
+        </is>
+      </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>2.0</t>
         </is>
       </c>
     </row>
@@ -894,25 +954,49 @@
           <t>Controller</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>4139.0</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>2.2</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>0.4363323152065277</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>0.2617993950843811</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>0xFFFC 0x0002</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr"/>
+          <t>65014.0</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>-522.0</t>
+        </is>
+      </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -962,25 +1046,41 @@
           <t>Controller</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>4139.0</t>
+        </is>
+      </c>
       <c r="K8" t="inlineStr">
         <is>
           <t>1.3</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>0xFFFC 0x0002</t>
-        </is>
-      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>0.4363323152065277</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>0.2617993950843811</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>2.0</t>
         </is>
       </c>
     </row>
@@ -1030,25 +1130,49 @@
           <t>Controller</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>4139.0</t>
+        </is>
+      </c>
       <c r="K9" t="inlineStr">
         <is>
           <t>2.3</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>0.4363323152065277</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>0.2617993950843811</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>0xFFFC 0x0002</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr"/>
+          <t>65014.0</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>-522.0</t>
+        </is>
+      </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -1098,25 +1222,49 @@
           <t>Controller</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>4139.0</t>
+        </is>
+      </c>
       <c r="K10" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>0.4363323152065277</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>0.2617993950843811</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>0xFFFC 0x0002</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr"/>
+          <t>65014.0</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>-522.0</t>
+        </is>
+      </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -1166,25 +1314,49 @@
           <t>Controller</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>3627.0</t>
+        </is>
+      </c>
       <c r="K11" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>0.4363323152065277</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>0.2617993950843811</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>0xFFFC 0x0002</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr"/>
+          <t>65014.0</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>-522.0</t>
+        </is>
+      </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>2.0</t>
         </is>
       </c>
     </row>
@@ -1242,17 +1414,21 @@
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>0xFFFC 0x0002</t>
-        </is>
-      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>-522.1</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>2.0</t>
         </is>
       </c>
     </row>
@@ -1302,25 +1478,49 @@
           <t>Controller</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>4139.0</t>
+        </is>
+      </c>
       <c r="K13" t="inlineStr">
         <is>
           <t>2.5</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>0.4363323152065277</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>0.2617993950843811</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>0xFFFC 0x0002</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr"/>
+          <t>65014.0</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>-522.0</t>
+        </is>
+      </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -1370,25 +1570,49 @@
           <t>Controller</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>4139.0</t>
+        </is>
+      </c>
       <c r="K14" t="inlineStr">
         <is>
           <t>1.6</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>0.4363323152065277</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>0.2617993950843811</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>0.12</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>0xFFFC 0x0002</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr"/>
+          <t>65014.0</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>-522.0</t>
+        </is>
+      </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -1438,25 +1662,49 @@
           <t>Controller</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>2603.0</t>
+        </is>
+      </c>
       <c r="K15" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>0.4363323152065277</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>0.2617993950843811</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>0xFFFC 0x0002</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr"/>
+          <t>65014.0</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>-522.0</t>
+        </is>
+      </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -1506,25 +1754,49 @@
           <t>Controller</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>4139.0</t>
+        </is>
+      </c>
       <c r="K16" t="inlineStr">
         <is>
           <t>1.7</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>0.4363323152065277</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>0.2617993950843811</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>0xFFFC 0x0002</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr"/>
+          <t>65014.0</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>-522.0</t>
+        </is>
+      </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -1582,17 +1854,21 @@
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>0xFFFC 0x0002</t>
-        </is>
-      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>-522.15</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>3.0</t>
         </is>
       </c>
     </row>
@@ -1650,17 +1926,21 @@
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>0xFFFC 0x0002</t>
-        </is>
-      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>0.16</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>-522.16</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>2.0</t>
         </is>
       </c>
     </row>
@@ -1718,17 +1998,21 @@
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>0xFFFC 0x0002</t>
-        </is>
-      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>0.17</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>-522.17</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>2.0</t>
         </is>
       </c>
     </row>
@@ -1786,17 +2070,21 @@
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>0xFFFC 0x0002</t>
-        </is>
-      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>0.18</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>-522.18</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>2.0</t>
         </is>
       </c>
     </row>
@@ -1846,38 +2134,14 @@
           <t>Meteo</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>5892.0</t>
-        </is>
-      </c>
+      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>8523.0</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>198.0</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>10289.0</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>62464.0</t>
-        </is>
-      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>0xFFDF 0x0000</t>
-        </is>
-      </c>
+      <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
           <t>1.0</t>

</xml_diff>

<commit_message>
3 fix read devices secuentialy not all the request at once (#4)
Read TSCs sequentially. Read just one register and move to the next device. This eliminates the possible swapping.
It also includes the save in NVM after the writings.

* Sequential

* Save NVM

---------

Co-authored-by: Aoyaga <Aoyaga@LT-ES-PF571D1J>
</commit_message>
<xml_diff>
--- a/config/Map_Escepar_1729509304301.xlsx
+++ b/config/Map_Escepar_1729509304301.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R21"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,40 +469,25 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>Write_41137</t>
+          <t>ReadF32_41044</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>ReadF32_41044</t>
+          <t>WriteF32_41048</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>ReadF32_41046</t>
+          <t>WriteS16_41050</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>WriteF32_41048</t>
+          <t>Mask_40000</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
-        <is>
-          <t>Write_41050</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>Read_41050</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>ReadS16_41050</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
         <is>
           <t>Attempts</t>
         </is>
@@ -546,7 +531,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>225</t>
+          <t>155</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -555,28 +540,25 @@
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>-522.0</t>
+        </is>
+      </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>0xFFFC 0x0002</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-522.0</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>3.0</t>
+          <t>2.0</t>
         </is>
       </c>
     </row>
@@ -618,7 +600,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>226</t>
+          <t>156</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -627,28 +609,25 @@
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>-522.1</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0xFFFC 0x0002</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
         <is>
           <t>2.0</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>-522.1</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>3.0</t>
         </is>
       </c>
     </row>
@@ -705,17 +684,17 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>0.4363323152065277</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0.4363323152065277</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>0.2617993950843811</t>
+          <t>-522.2</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -724,21 +703,6 @@
         </is>
       </c>
       <c r="O4" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>65014.0</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>-522.0</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
@@ -791,26 +755,23 @@
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>2.1</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>-522.3</t>
+        </is>
+      </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>0xFFFC 0x0002</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
-        <is>
-          <t>-522.3</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr">
         <is>
           <t>2.0</t>
         </is>
@@ -869,17 +830,17 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>0.4363323152065277</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2.169474251394558e-19</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2.169474251394558e-19</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -889,22 +850,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>4139.0</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>26355.0</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>2.0</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -961,17 +907,17 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>0.4363323152065277</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0.4363323152065277</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>0.2617993950843811</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -980,21 +926,6 @@
         </is>
       </c>
       <c r="O7" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>65014.0</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>-522.0</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
@@ -1053,17 +984,17 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>0.4363323152065277</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0.4363323152065277</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>0.2617993950843811</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1073,14 +1004,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>2.0</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -1137,17 +1061,17 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>0.4363323152065277</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0.4363323152065277</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>0.2617993950843811</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1156,21 +1080,6 @@
         </is>
       </c>
       <c r="O9" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>65014.0</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>-522.0</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
@@ -1229,40 +1138,25 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>0.4363323152065277</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0.4363323152065277</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>0.2617993950843811</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>65014.0</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>-522.0</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
@@ -1321,42 +1215,27 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>0.4363323152065277</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0.4363323152065277</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>0.2617993950843811</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>0.9</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>65014.0</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>-522.0</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>2.0</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -1407,28 +1286,25 @@
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>1.5</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>-522.1</t>
+        </is>
+      </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>0xFFFC 0x0002</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>-522.1</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>2.0</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -1485,17 +1361,17 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>0.4363323152065277</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0.4363323152065277</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>0.2617993950843811</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1504,21 +1380,6 @@
         </is>
       </c>
       <c r="O13" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>65014.0</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>-522.0</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
@@ -1577,40 +1438,25 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>0.4363323152065277</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0.4363323152065277</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>0.2617993950843811</t>
+          <t>-522.12</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>0.12</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>65014.0</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>-522.0</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
@@ -1669,40 +1515,25 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2.6</t>
+          <t>0.4363323152065277</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0.4363323152065277</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>0.2617993950843811</t>
+          <t>-522.13</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>0xFFFC 0x0002</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>65014.0</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>-522.0</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
@@ -1761,17 +1592,17 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>0.4363323152065277</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0.4363323152065277</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>0.2617993950843811</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1780,21 +1611,6 @@
         </is>
       </c>
       <c r="O16" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>65014.0</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>-522.0</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
@@ -1847,28 +1663,25 @@
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>2.7</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>-522.15</t>
+        </is>
+      </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>0.15</t>
+          <t>0xFFFC 0x0002</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>-522.15</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>3.0</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -1919,28 +1732,25 @@
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>1.8</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>0.16</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>-522.16</t>
+        </is>
+      </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>0.16</t>
+          <t>0xFFFC 0x0002</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>-522.16</t>
-        </is>
-      </c>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>2.0</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -1991,28 +1801,25 @@
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>2.8</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>0.17</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>-522.17</t>
+        </is>
+      </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>0.17</t>
+          <t>0xFFFC 0x0002</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>-522.17</t>
-        </is>
-      </c>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>2.0</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -2063,28 +1870,25 @@
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>1.9</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>0.18</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>-522.18</t>
+        </is>
+      </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>0.18</t>
+          <t>0xFFFC 0x0002</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>-522.18</t>
-        </is>
-      </c>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>2.0</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -2139,10 +1943,7 @@
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>

</xml_diff>